<commit_message>
Update data from new Excel workbook (VBOS Section BP_2026)
</commit_message>
<xml_diff>
--- a/data/VBOS-Section-BP_2026.xlsx
+++ b/data/VBOS-Section-BP_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29926"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30023"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\achilia\Documents\Vanuatu Bureau of Statistics Files\VBoS Business Plan\2026 VBoS Business Plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A2B76B20-F322-41FF-89C9-4295FF8E0B21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="282" documentId="11_D6403AD3BB22401C7C3FEE499908F29706559575" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{715E666D-5F51-42D3-A246-6A2219B901FF}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1601-CS Office" sheetId="9" r:id="rId1"/>
@@ -271,118 +271,118 @@
     <t>2024-2025 Labour Force Survey</t>
   </si>
   <si>
+    <t>In progress</t>
+  </si>
+  <si>
+    <t>HIES</t>
+  </si>
+  <si>
+    <t>2.1.2.. Training of Trainers</t>
+  </si>
+  <si>
+    <t>2025 HIES</t>
+  </si>
+  <si>
+    <t>2026-2027</t>
+  </si>
+  <si>
+    <t>1. Natural Disaster (Cyclone Season)</t>
+  </si>
+  <si>
+    <t>Complete</t>
+  </si>
+  <si>
+    <t>2.1.3. Training of Enumerator</t>
+  </si>
+  <si>
+    <t>Assist Port Vila</t>
+  </si>
+  <si>
+    <t>2. Enumerator Turnover</t>
+  </si>
+  <si>
+    <t>2.1.4.. Fieldwork Monitoring of Enumerators</t>
+  </si>
+  <si>
+    <t>3. Delay of Funds</t>
+  </si>
+  <si>
+    <t>NCD SURVEY</t>
+  </si>
+  <si>
+    <t>2.1.5. Provide Technical Support</t>
+  </si>
+  <si>
+    <t>Field work collection monitoring in Sanma</t>
+  </si>
+  <si>
+    <t>Production of Regular Pulbications</t>
+  </si>
+  <si>
+    <t>CPI</t>
+  </si>
+  <si>
+    <t>2.2.1. 26 Data Collection &amp; 26 Entries</t>
+  </si>
+  <si>
+    <t>CPI Forhtnighly Data Collection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Delay in prining </t>
+  </si>
+  <si>
+    <t>2.2.2. 4 Data Collection</t>
+  </si>
+  <si>
+    <t>CPI Quaterly Data Collection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. No available vehicle </t>
+  </si>
+  <si>
+    <t>3. Unforseen circumstances</t>
+  </si>
+  <si>
+    <t>MARKET SURVEY</t>
+  </si>
+  <si>
+    <t>2.2.3. 26 Data Collection &amp; 26 Entries</t>
+  </si>
+  <si>
+    <t>Market Survey Fornightly Data Collection &amp; Entry</t>
+  </si>
+  <si>
+    <t>PROVINCIAL REPORTS</t>
+  </si>
+  <si>
+    <t>2.3.4. Provincial Statistical Indicator- (PSI)</t>
+  </si>
+  <si>
+    <t>DCM Reporting and Development</t>
+  </si>
+  <si>
+    <t>STAFF WORKPLAN</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2.3.1. Annual long-term goals with monthly reviews</t>
+  </si>
+  <si>
+    <t>DCM Staff Monthly Reporting</t>
+  </si>
+  <si>
+    <t>QUATERLY SECTION MEETINGS</t>
+  </si>
+  <si>
+    <t>2.3.2. DCM Quaterly Section Meetings</t>
+  </si>
+  <si>
+    <t>CAPACITY BUILDING</t>
+  </si>
+  <si>
+    <t>2.3.3. Capacity Building for DCM Staffs through online, in-house and external trainings. (Survey Solutions, Tableau, R)</t>
+  </si>
+  <si>
     <t>Not yet Started</t>
-  </si>
-  <si>
-    <t>HIES</t>
-  </si>
-  <si>
-    <t>2.1.2.. Training of Trainers</t>
-  </si>
-  <si>
-    <t>2025 HIES</t>
-  </si>
-  <si>
-    <t>2026-2027</t>
-  </si>
-  <si>
-    <t>1. Natural Disaster (Cyclone Season)</t>
-  </si>
-  <si>
-    <t>Complete</t>
-  </si>
-  <si>
-    <t>2.1.3. Training of Enumerator</t>
-  </si>
-  <si>
-    <t>Assist Port Vila</t>
-  </si>
-  <si>
-    <t>2. Enumerator Turnover</t>
-  </si>
-  <si>
-    <t>2.1.4.. Fieldwork Monitoring of Enumerators</t>
-  </si>
-  <si>
-    <t>3. Delay of Funds</t>
-  </si>
-  <si>
-    <t>In progress</t>
-  </si>
-  <si>
-    <t>NCD SURVEY</t>
-  </si>
-  <si>
-    <t>2.1.5. Provide Technical Support</t>
-  </si>
-  <si>
-    <t>Field work collection monitoring in Sanma</t>
-  </si>
-  <si>
-    <t>Production of Regular Pulbications</t>
-  </si>
-  <si>
-    <t>CPI</t>
-  </si>
-  <si>
-    <t>2.2.1. 26 Data Collection &amp; 26 Entries</t>
-  </si>
-  <si>
-    <t>CPI Forhtnighly Data Collection</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Delay in prining </t>
-  </si>
-  <si>
-    <t>2.2.2. 4 Data Collection</t>
-  </si>
-  <si>
-    <t>CPI Quaterly Data Collection</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. No available vehicle </t>
-  </si>
-  <si>
-    <t>3. Unforseen circumstances</t>
-  </si>
-  <si>
-    <t>MARKET SURVEY</t>
-  </si>
-  <si>
-    <t>2.2.3. 26 Data Collection &amp; 26 Entries</t>
-  </si>
-  <si>
-    <t>Market Survey Fornightly Data Collection &amp; Entry</t>
-  </si>
-  <si>
-    <t>PROVINCIAL REPORTS</t>
-  </si>
-  <si>
-    <t>2.3.4. Provincial Statistical Indicator- (PSI)</t>
-  </si>
-  <si>
-    <t>DCM Reporting and Development</t>
-  </si>
-  <si>
-    <t>STAFF WORKPLAN</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 2.3.1. Annual long-term goals with monthly reviews</t>
-  </si>
-  <si>
-    <t>DCM Staff Monthly Reporting</t>
-  </si>
-  <si>
-    <t>QUATERLY SECTION MEETINGS</t>
-  </si>
-  <si>
-    <t>2.3.2. DCM Quaterly Section Meetings</t>
-  </si>
-  <si>
-    <t>CAPACITY BUILDING</t>
-  </si>
-  <si>
-    <t>2.3.3. Capacity Building for DCM Staffs through online, in-house and external trainings. (Survey Solutions, Tableau, R)</t>
   </si>
   <si>
     <t>QUATERLY REPORTING TO CS OFFICE</t>
@@ -11755,7 +11755,7 @@
       </c>
       <c r="E8" s="621"/>
       <c r="F8" s="609" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G8" s="569"/>
       <c r="H8" s="570"/>
@@ -12428,7 +12428,7 @@
         <v>85</v>
       </c>
       <c r="K7" s="470" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -12440,7 +12440,7 @@
         <v>69</v>
       </c>
       <c r="F8" s="471" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G8" s="435"/>
       <c r="H8" s="436"/>
@@ -12455,20 +12455,20 @@
       <c r="D9" s="1330"/>
       <c r="E9" s="1348"/>
       <c r="F9" s="382" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G9" s="474">
         <v>1</v>
       </c>
       <c r="H9" s="382" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I9" s="475">
         <v>2026</v>
       </c>
       <c r="J9" s="476"/>
       <c r="K9" s="477" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -12477,7 +12477,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="C10" s="1303" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D10" s="1300" t="s">
         <v>68</v>
@@ -12486,7 +12486,7 @@
         <v>500000</v>
       </c>
       <c r="F10" s="463" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G10" s="457"/>
       <c r="H10" s="386"/>
@@ -12501,20 +12501,20 @@
       <c r="D11" s="1301"/>
       <c r="E11" s="1313"/>
       <c r="F11" s="424" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G11" s="212">
         <v>26</v>
       </c>
       <c r="H11" s="424" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="I11" s="425"/>
       <c r="J11" s="84" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="K11" s="444" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -12524,22 +12524,22 @@
       <c r="D12" s="1301"/>
       <c r="E12" s="1313"/>
       <c r="F12" s="1345" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G12" s="1352">
         <v>4</v>
       </c>
       <c r="H12" s="1345" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I12" s="425">
         <v>46387</v>
       </c>
       <c r="J12" s="84" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="K12" s="1350" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="14.45" customHeight="1" thickBot="1">
@@ -12553,7 +12553,7 @@
       <c r="H13" s="1346"/>
       <c r="I13" s="35"/>
       <c r="J13" s="446" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="K13" s="1351"/>
     </row>
@@ -12564,7 +12564,7 @@
       <c r="D14" s="1301"/>
       <c r="E14" s="1315"/>
       <c r="F14" s="478" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G14" s="421"/>
       <c r="H14" s="451"/>
@@ -12579,20 +12579,20 @@
       <c r="D15" s="1301"/>
       <c r="E15" s="1316"/>
       <c r="F15" s="446" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G15" s="213">
         <v>26</v>
       </c>
       <c r="H15" s="446" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I15" s="447">
         <v>46387</v>
       </c>
       <c r="J15" s="446"/>
       <c r="K15" s="448" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -12604,7 +12604,7 @@
         <v>100000</v>
       </c>
       <c r="F16" s="454" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G16" s="455"/>
       <c r="H16" s="453"/>
@@ -12619,7 +12619,7 @@
       <c r="D17" s="1302"/>
       <c r="E17" s="1316"/>
       <c r="F17" s="446" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G17" s="213">
         <v>6</v>
@@ -12630,7 +12630,7 @@
       </c>
       <c r="J17" s="446"/>
       <c r="K17" s="448" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -12639,14 +12639,14 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="C18" s="1297" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D18" s="1318" t="s">
         <v>68</v>
       </c>
       <c r="E18" s="1357"/>
       <c r="F18" s="482" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G18" s="483"/>
       <c r="H18" s="484"/>
@@ -12661,20 +12661,20 @@
       <c r="D19" s="1319"/>
       <c r="E19" s="1358"/>
       <c r="F19" s="489" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G19" s="490">
         <v>12</v>
       </c>
       <c r="H19" s="489" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I19" s="491">
         <v>46387</v>
       </c>
       <c r="J19" s="489"/>
       <c r="K19" s="492" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -12686,7 +12686,7 @@
         <v>100000</v>
       </c>
       <c r="F20" s="482" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G20" s="483"/>
       <c r="H20" s="484"/>
@@ -12701,7 +12701,7 @@
       <c r="D21" s="1319"/>
       <c r="E21" s="1358"/>
       <c r="F21" s="489" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G21" s="490">
         <v>4</v>
@@ -12724,7 +12724,7 @@
         <v>200000</v>
       </c>
       <c r="F22" s="482" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G22" s="483"/>
       <c r="H22" s="484"/>
@@ -12739,7 +12739,7 @@
       <c r="D23" s="1319"/>
       <c r="E23" s="1358"/>
       <c r="F23" s="489" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G23" s="490">
         <v>4</v>
@@ -12750,7 +12750,7 @@
       </c>
       <c r="J23" s="489"/>
       <c r="K23" s="492" t="s">
-        <v>74</v>
+        <v>111</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -12786,7 +12786,7 @@
       </c>
       <c r="J25" s="489"/>
       <c r="K25" s="492" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="14.45" customHeight="1">
@@ -12815,7 +12815,7 @@
       </c>
       <c r="J26" s="494"/>
       <c r="K26" s="497" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="15">
@@ -12836,7 +12836,7 @@
       </c>
       <c r="J27" s="8"/>
       <c r="K27" s="498" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="15">
@@ -12857,7 +12857,7 @@
       </c>
       <c r="J28" s="8"/>
       <c r="K28" s="498" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="15">
@@ -12878,7 +12878,7 @@
       </c>
       <c r="J29" s="8"/>
       <c r="K29" s="498" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="15" thickBot="1">
@@ -12899,7 +12899,7 @@
       </c>
       <c r="J30" s="9"/>
       <c r="K30" s="499" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="27.75">
@@ -12926,7 +12926,7 @@
       </c>
       <c r="J31" s="74"/>
       <c r="K31" s="504" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="27.75">
@@ -12947,7 +12947,7 @@
       <c r="I32" s="76"/>
       <c r="J32" s="502"/>
       <c r="K32" s="505" t="s">
-        <v>74</v>
+        <v>111</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="34.15" customHeight="1" thickBot="1">
@@ -12966,7 +12966,7 @@
       <c r="I33" s="81"/>
       <c r="J33" s="127"/>
       <c r="K33" s="506" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
     </row>
     <row r="34" spans="1:11" ht="15" thickBot="1">
@@ -19541,7 +19541,7 @@
         <v>1</v>
       </c>
       <c r="H7" s="533" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I7" s="1803"/>
       <c r="J7" s="586"/>
@@ -19560,7 +19560,7 @@
       </c>
       <c r="E8" s="621"/>
       <c r="F8" s="609" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G8" s="569"/>
       <c r="H8" s="570"/>
@@ -20624,15 +20624,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <SharedWithUsers xmlns="a521bc18-84a4-4135-8fab-fb26feb7c8d1">
@@ -20650,7 +20641,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010050A54B94194EE0459E0DF1A0F18383A4" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ef292490ca0b79147bc159b72553183c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="496a2456-8dd7-43f2-a878-9b7aec5435e7" xmlns:ns3="a521bc18-84a4-4135-8fab-fb26feb7c8d1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b93ed5a678b854dfcaa98bc235cc39ba" ns2:_="" ns3:_="">
     <xsd:import namespace="496a2456-8dd7-43f2-a878-9b7aec5435e7"/>
@@ -20873,14 +20864,23 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E6BC0936-C675-45B7-83CC-DDA638FB0D73}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A5D6C6A-D9A7-452D-A82A-3D5B1917D942}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A5D6C6A-D9A7-452D-A82A-3D5B1917D942}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CE7CB1BB-04C5-4906-B8A2-C9FE087589FC}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CE7CB1BB-04C5-4906-B8A2-C9FE087589FC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E6BC0936-C675-45B7-83CC-DDA638FB0D73}"/>
 </file>
</xml_diff>